<commit_message>
Add Top 150 Keywords sheet to content master Excel
150 niche keywords organized by search intent (Informational/Commercial/Navigational),
funnel stage (Top/Mid/Bottom), and priority (P1-P3) with notes on strategic value.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bioskinrepair-content-master.xlsx
+++ b/bioskinrepair-content-master.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content Inventory" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top 150 Keywords" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Content Inventory'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Top 150 Keywords'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -108,6 +110,43 @@
       <color rgb="004A148C"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00999999"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00111111"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00E65100"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00666666"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001565C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="002E7D32"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00757575"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -158,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -252,6 +291,72 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2404,6 +2509,4105 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F151"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Keyword</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Search Intent</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Funnel Stage</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier repair</t>
+        </is>
+      </c>
+      <c r="C2" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D2" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E2" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F2" s="37" t="inlineStr">
+        <is>
+          <t>Primary niche keyword</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier</t>
+        </is>
+      </c>
+      <c r="C3" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D3" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E3" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F3" s="43" t="inlineStr">
+        <is>
+          <t>Broadest head term</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="32" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C4" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F4" s="37" t="inlineStr">
+        <is>
+          <t>High volume intent to learn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>how to repair skin barrier</t>
+        </is>
+      </c>
+      <c r="C5" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D5" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E5" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F5" s="43" t="inlineStr">
+        <is>
+          <t>Top how-to query</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="32" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier function</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D6" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F6" s="37" t="inlineStr">
+        <is>
+          <t>Educational intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="39" t="inlineStr">
+        <is>
+          <t>what is the skin barrier</t>
+        </is>
+      </c>
+      <c r="C7" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F7" s="43" t="inlineStr">
+        <is>
+          <t>TOFU educational</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="32" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier damage symptoms</t>
+        </is>
+      </c>
+      <c r="C8" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F8" s="37" t="inlineStr">
+        <is>
+          <t>Problem-aware user</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>how to fix damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D9" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F9" s="43" t="inlineStr">
+        <is>
+          <t>Action intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="32" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier recovery</t>
+        </is>
+      </c>
+      <c r="C10" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D10" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E10" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F10" s="37" t="inlineStr">
+        <is>
+          <t>Recovery phase</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>restore skin barrier</t>
+        </is>
+      </c>
+      <c r="C11" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E11" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F11" s="43" t="inlineStr">
+        <is>
+          <t>Active repair intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="32" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="33" t="inlineStr">
+        <is>
+          <t>how long does skin barrier take to heal</t>
+        </is>
+      </c>
+      <c r="C12" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D12" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E12" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F12" s="37" t="inlineStr">
+        <is>
+          <t>High commercial &amp; info overlap</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="38" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="39" t="inlineStr">
+        <is>
+          <t>signs skin barrier is healing</t>
+        </is>
+      </c>
+      <c r="C13" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D13" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F13" s="43" t="inlineStr">
+        <is>
+          <t>Progress checker</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier repair timeline</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D14" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F14" s="37" t="inlineStr"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="38" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="39" t="inlineStr">
+        <is>
+          <t>how to speed up skin barrier repair</t>
+        </is>
+      </c>
+      <c r="C15" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D15" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E15" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F15" s="43" t="inlineStr">
+        <is>
+          <t>High intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="32" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="33" t="inlineStr">
+        <is>
+          <t>why does skin feel tight</t>
+        </is>
+      </c>
+      <c r="C16" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D16" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E16" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F16" s="37" t="inlineStr">
+        <is>
+          <t>Symptom-led entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="39" t="inlineStr">
+        <is>
+          <t>why is my skin flaky</t>
+        </is>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D17" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E17" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F17" s="43" t="inlineStr">
+        <is>
+          <t>Symptom-led entry</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="32" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier compromised</t>
+        </is>
+      </c>
+      <c r="C18" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D18" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E18" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F18" s="37" t="inlineStr"/>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="38" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>how to tell if skin barrier is damaged</t>
+        </is>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D19" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E19" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F19" s="43" t="inlineStr">
+        <is>
+          <t>Diagnosis intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="32" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier healing signs week by week</t>
+        </is>
+      </c>
+      <c r="C20" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D20" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E20" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F20" s="37" t="inlineStr"/>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier still damaged after weeks</t>
+        </is>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D21" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E21" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F21" s="43" t="inlineStr">
+        <is>
+          <t>Frustrated user</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="32" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="33" t="inlineStr">
+        <is>
+          <t>ceramides for skin</t>
+        </is>
+      </c>
+      <c r="C22" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D22" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E22" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F22" s="37" t="inlineStr">
+        <is>
+          <t>Core ingredient term</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="38" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="39" t="inlineStr">
+        <is>
+          <t>ceramide moisturizer</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D23" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E23" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F23" s="43" t="inlineStr">
+        <is>
+          <t>Buying intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="32" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="33" t="inlineStr">
+        <is>
+          <t>best ceramide moisturizer</t>
+        </is>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D24" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E24" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F24" s="37" t="inlineStr">
+        <is>
+          <t>High purchase intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="38" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="39" t="inlineStr">
+        <is>
+          <t>ceramide cream for dry skin</t>
+        </is>
+      </c>
+      <c r="C25" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D25" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E25" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F25" s="43" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="32" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="33" t="inlineStr">
+        <is>
+          <t>what do ceramides do for skin</t>
+        </is>
+      </c>
+      <c r="C26" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D26" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F26" s="37" t="inlineStr"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="38" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="39" t="inlineStr">
+        <is>
+          <t>humectant skincare</t>
+        </is>
+      </c>
+      <c r="C27" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D27" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E27" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F27" s="43" t="inlineStr"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="32" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="33" t="inlineStr">
+        <is>
+          <t>what is a humectant</t>
+        </is>
+      </c>
+      <c r="C28" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D28" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E28" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F28" s="37" t="inlineStr"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="38" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="39" t="inlineStr">
+        <is>
+          <t>best humectant for dry skin</t>
+        </is>
+      </c>
+      <c r="C29" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D29" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E29" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F29" s="43" t="inlineStr"/>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="32" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="33" t="inlineStr">
+        <is>
+          <t>humectant vs emollient vs occlusive</t>
+        </is>
+      </c>
+      <c r="C30" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D30" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E30" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F30" s="37" t="inlineStr">
+        <is>
+          <t>Comparison intent</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="39" t="inlineStr">
+        <is>
+          <t>occlusive skincare</t>
+        </is>
+      </c>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D31" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E31" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F31" s="43" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="33" t="inlineStr">
+        <is>
+          <t>what is an occlusive</t>
+        </is>
+      </c>
+      <c r="C32" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D32" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E32" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F32" s="37" t="inlineStr"/>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="38" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="39" t="inlineStr">
+        <is>
+          <t>best occlusive moisturizer</t>
+        </is>
+      </c>
+      <c r="C33" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D33" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E33" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F33" s="43" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="32" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="33" t="inlineStr">
+        <is>
+          <t>occlusive for skin barrier</t>
+        </is>
+      </c>
+      <c r="C34" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D34" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E34" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F34" s="37" t="inlineStr"/>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="39" t="inlineStr">
+        <is>
+          <t>emollient skin</t>
+        </is>
+      </c>
+      <c r="C35" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D35" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E35" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F35" s="43" t="inlineStr"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="32" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="33" t="inlineStr">
+        <is>
+          <t>what is an emollient in skincare</t>
+        </is>
+      </c>
+      <c r="C36" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D36" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E36" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F36" s="37" t="inlineStr"/>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="39" t="inlineStr">
+        <is>
+          <t>emollient vs moisturizer</t>
+        </is>
+      </c>
+      <c r="C37" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D37" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E37" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F37" s="43" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="32" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="33" t="inlineStr">
+        <is>
+          <t>hyaluronic acid for skin barrier</t>
+        </is>
+      </c>
+      <c r="C38" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D38" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E38" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F38" s="37" t="inlineStr"/>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="38" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="39" t="inlineStr">
+        <is>
+          <t>hyaluronic acid dry skin</t>
+        </is>
+      </c>
+      <c r="C39" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D39" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E39" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F39" s="43" t="inlineStr"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="32" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="33" t="inlineStr">
+        <is>
+          <t>is hyaluronic acid good for damaged skin</t>
+        </is>
+      </c>
+      <c r="C40" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D40" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E40" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F40" s="37" t="inlineStr"/>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="38" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="39" t="inlineStr">
+        <is>
+          <t>niacinamide skin barrier</t>
+        </is>
+      </c>
+      <c r="C41" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D41" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E41" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F41" s="43" t="inlineStr"/>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="32" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="33" t="inlineStr">
+        <is>
+          <t>niacinamide for sensitive skin</t>
+        </is>
+      </c>
+      <c r="C42" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D42" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E42" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F42" s="37" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="38" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="39" t="inlineStr">
+        <is>
+          <t>glycerin for skin</t>
+        </is>
+      </c>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D43" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E43" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F43" s="43" t="inlineStr"/>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="32" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="33" t="inlineStr">
+        <is>
+          <t>glycerin vs hyaluronic acid</t>
+        </is>
+      </c>
+      <c r="C44" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D44" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E44" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F44" s="37" t="inlineStr"/>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="38" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="39" t="inlineStr">
+        <is>
+          <t>panthenol skincare</t>
+        </is>
+      </c>
+      <c r="C45" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E45" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F45" s="43" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="32" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="33" t="inlineStr">
+        <is>
+          <t>vitamin B5 skin</t>
+        </is>
+      </c>
+      <c r="C46" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D46" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E46" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F46" s="37" t="inlineStr"/>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="38" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="39" t="inlineStr">
+        <is>
+          <t>TEWL skin barrier</t>
+        </is>
+      </c>
+      <c r="C47" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E47" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F47" s="43" t="inlineStr">
+        <is>
+          <t>Niche technical term</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="32" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="33" t="inlineStr">
+        <is>
+          <t>transepidermal water loss</t>
+        </is>
+      </c>
+      <c r="C48" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D48" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E48" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F48" s="37" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="38" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="39" t="inlineStr">
+        <is>
+          <t>skincare routine for damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C49" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E49" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F49" s="43" t="inlineStr">
+        <is>
+          <t>High purchase proximity</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="32" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="33" t="inlineStr">
+        <is>
+          <t>minimalist skincare routine sensitive skin</t>
+        </is>
+      </c>
+      <c r="C50" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D50" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E50" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F50" s="37" t="inlineStr"/>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="38" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="39" t="inlineStr">
+        <is>
+          <t>simple skincare routine barrier repair</t>
+        </is>
+      </c>
+      <c r="C51" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D51" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E51" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F51" s="43" t="inlineStr"/>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="32" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="33" t="inlineStr">
+        <is>
+          <t>what not to use on damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C52" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D52" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E52" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F52" s="37" t="inlineStr">
+        <is>
+          <t>Negative intent — high click</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="38" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="39" t="inlineStr">
+        <is>
+          <t>skincare routine skin barrier recovery</t>
+        </is>
+      </c>
+      <c r="C53" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D53" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E53" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F53" s="43" t="inlineStr"/>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="32" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="33" t="inlineStr">
+        <is>
+          <t>how many products to use with damaged barrier</t>
+        </is>
+      </c>
+      <c r="C54" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D54" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E54" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F54" s="37" t="inlineStr"/>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="38" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="39" t="inlineStr">
+        <is>
+          <t>can you use retinol with damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D55" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E55" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F55" s="43" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="32" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="33" t="inlineStr">
+        <is>
+          <t>how to layer skincare products</t>
+        </is>
+      </c>
+      <c r="C56" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D56" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E56" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F56" s="37" t="inlineStr"/>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="38" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="39" t="inlineStr">
+        <is>
+          <t>over exfoliation</t>
+        </is>
+      </c>
+      <c r="C57" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D57" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E57" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F57" s="43" t="inlineStr">
+        <is>
+          <t>High volume problem query</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="32" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="33" t="inlineStr">
+        <is>
+          <t>signs of over exfoliated skin</t>
+        </is>
+      </c>
+      <c r="C58" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D58" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E58" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F58" s="37" t="inlineStr"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="38" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="39" t="inlineStr">
+        <is>
+          <t>how to recover from over exfoliation</t>
+        </is>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D59" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E59" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F59" s="43" t="inlineStr"/>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="32" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="33" t="inlineStr">
+        <is>
+          <t>over exfoliation recovery routine</t>
+        </is>
+      </c>
+      <c r="C60" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D60" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E60" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F60" s="37" t="inlineStr"/>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="38" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="39" t="inlineStr">
+        <is>
+          <t>AHA vs BHA sensitive skin</t>
+        </is>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D61" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E61" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F61" s="43" t="inlineStr"/>
+    </row>
+    <row r="62" ht="18" customHeight="1">
+      <c r="A62" s="32" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="33" t="inlineStr">
+        <is>
+          <t>chemical exfoliant damaged barrier</t>
+        </is>
+      </c>
+      <c r="C62" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D62" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E62" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F62" s="37" t="inlineStr"/>
+    </row>
+    <row r="63" ht="18" customHeight="1">
+      <c r="A63" s="38" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="39" t="inlineStr">
+        <is>
+          <t>how often to exfoliate sensitive skin</t>
+        </is>
+      </c>
+      <c r="C63" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D63" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E63" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F63" s="43" t="inlineStr"/>
+    </row>
+    <row r="64" ht="18" customHeight="1">
+      <c r="A64" s="32" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="33" t="inlineStr">
+        <is>
+          <t>retinol skin barrier damage</t>
+        </is>
+      </c>
+      <c r="C64" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D64" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E64" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F64" s="37" t="inlineStr"/>
+    </row>
+    <row r="65" ht="18" customHeight="1">
+      <c r="A65" s="38" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="39" t="inlineStr">
+        <is>
+          <t>does retinol damage skin barrier</t>
+        </is>
+      </c>
+      <c r="C65" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D65" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E65" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F65" s="43" t="inlineStr"/>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="32" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="33" t="inlineStr">
+        <is>
+          <t>retinol for beginners sensitive skin</t>
+        </is>
+      </c>
+      <c r="C66" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D66" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E66" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F66" s="37" t="inlineStr"/>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="38" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="39" t="inlineStr">
+        <is>
+          <t>how to use retinol without irritation</t>
+        </is>
+      </c>
+      <c r="C67" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D67" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E67" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F67" s="43" t="inlineStr"/>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="32" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="33" t="inlineStr">
+        <is>
+          <t>retinol purging vs barrier damage</t>
+        </is>
+      </c>
+      <c r="C68" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D68" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E68" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F68" s="37" t="inlineStr"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="38" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="39" t="inlineStr">
+        <is>
+          <t>when to stop retinol skin barrier</t>
+        </is>
+      </c>
+      <c r="C69" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D69" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E69" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F69" s="43" t="inlineStr"/>
+    </row>
+    <row r="70" ht="18" customHeight="1">
+      <c r="A70" s="32" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="33" t="inlineStr">
+        <is>
+          <t>mineral vs chemical sunscreen</t>
+        </is>
+      </c>
+      <c r="C70" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D70" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E70" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F70" s="37" t="inlineStr"/>
+    </row>
+    <row r="71" ht="18" customHeight="1">
+      <c r="A71" s="38" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="39" t="inlineStr">
+        <is>
+          <t>best sunscreen for sensitive skin</t>
+        </is>
+      </c>
+      <c r="C71" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D71" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E71" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F71" s="43" t="inlineStr"/>
+    </row>
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="32" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="33" t="inlineStr">
+        <is>
+          <t>mineral sunscreen for damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C72" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D72" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E72" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F72" s="37" t="inlineStr"/>
+    </row>
+    <row r="73" ht="18" customHeight="1">
+      <c r="A73" s="38" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="39" t="inlineStr">
+        <is>
+          <t>does sunscreen irritate sensitive skin</t>
+        </is>
+      </c>
+      <c r="C73" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D73" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E73" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F73" s="43" t="inlineStr"/>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="32" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="33" t="inlineStr">
+        <is>
+          <t>zinc oxide sunscreen sensitive skin</t>
+        </is>
+      </c>
+      <c r="C74" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D74" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E74" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F74" s="37" t="inlineStr"/>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="38" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="39" t="inlineStr">
+        <is>
+          <t>sunscreen for skin barrier repair</t>
+        </is>
+      </c>
+      <c r="C75" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D75" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E75" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F75" s="43" t="inlineStr"/>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="32" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="33" t="inlineStr">
+        <is>
+          <t>EltaMD UV Clear review</t>
+        </is>
+      </c>
+      <c r="C76" s="50" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D76" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E76" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F76" s="37" t="inlineStr"/>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="38" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="39" t="inlineStr">
+        <is>
+          <t>eczema skin barrier</t>
+        </is>
+      </c>
+      <c r="C77" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D77" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E77" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F77" s="43" t="inlineStr"/>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="32" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="33" t="inlineStr">
+        <is>
+          <t>eczema barrier repair</t>
+        </is>
+      </c>
+      <c r="C78" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D78" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E78" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F78" s="37" t="inlineStr"/>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="38" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="39" t="inlineStr">
+        <is>
+          <t>best moisturizer for eczema</t>
+        </is>
+      </c>
+      <c r="C79" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D79" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E79" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F79" s="43" t="inlineStr"/>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="32" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="33" t="inlineStr">
+        <is>
+          <t>ceramides for eczema</t>
+        </is>
+      </c>
+      <c r="C80" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D80" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E80" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F80" s="37" t="inlineStr"/>
+    </row>
+    <row r="81" ht="18" customHeight="1">
+      <c r="A81" s="38" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="39" t="inlineStr">
+        <is>
+          <t>eczema skincare routine</t>
+        </is>
+      </c>
+      <c r="C81" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D81" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E81" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F81" s="43" t="inlineStr"/>
+    </row>
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="32" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="33" t="inlineStr">
+        <is>
+          <t>what causes eczema flares</t>
+        </is>
+      </c>
+      <c r="C82" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D82" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E82" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F82" s="37" t="inlineStr"/>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="38" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="39" t="inlineStr">
+        <is>
+          <t>rosacea skin barrier</t>
+        </is>
+      </c>
+      <c r="C83" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D83" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E83" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F83" s="43" t="inlineStr"/>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="32" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="33" t="inlineStr">
+        <is>
+          <t>best moisturizer for rosacea</t>
+        </is>
+      </c>
+      <c r="C84" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D84" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E84" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F84" s="37" t="inlineStr"/>
+    </row>
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="38" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="39" t="inlineStr">
+        <is>
+          <t>rosacea skincare routine</t>
+        </is>
+      </c>
+      <c r="C85" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D85" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E85" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F85" s="43" t="inlineStr"/>
+    </row>
+    <row r="86" ht="18" customHeight="1">
+      <c r="A86" s="32" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="33" t="inlineStr">
+        <is>
+          <t>does rosacea damage skin barrier</t>
+        </is>
+      </c>
+      <c r="C86" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D86" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E86" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F86" s="37" t="inlineStr"/>
+    </row>
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="38" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="39" t="inlineStr">
+        <is>
+          <t>rosacea barrier repair routine</t>
+        </is>
+      </c>
+      <c r="C87" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D87" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E87" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F87" s="43" t="inlineStr"/>
+    </row>
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="32" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="33" t="inlineStr">
+        <is>
+          <t>perioral dermatitis</t>
+        </is>
+      </c>
+      <c r="C88" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D88" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E88" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F88" s="37" t="inlineStr"/>
+    </row>
+    <row r="89" ht="18" customHeight="1">
+      <c r="A89" s="38" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="39" t="inlineStr">
+        <is>
+          <t>perioral dermatitis causes</t>
+        </is>
+      </c>
+      <c r="C89" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D89" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E89" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F89" s="43" t="inlineStr"/>
+    </row>
+    <row r="90" ht="18" customHeight="1">
+      <c r="A90" s="32" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="33" t="inlineStr">
+        <is>
+          <t>perioral dermatitis treatment</t>
+        </is>
+      </c>
+      <c r="C90" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D90" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E90" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F90" s="37" t="inlineStr"/>
+    </row>
+    <row r="91" ht="18" customHeight="1">
+      <c r="A91" s="38" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="39" t="inlineStr">
+        <is>
+          <t>how to clear perioral dermatitis</t>
+        </is>
+      </c>
+      <c r="C91" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D91" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E91" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F91" s="43" t="inlineStr"/>
+    </row>
+    <row r="92" ht="18" customHeight="1">
+      <c r="A92" s="32" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="33" t="inlineStr">
+        <is>
+          <t>perioral dermatitis skincare routine</t>
+        </is>
+      </c>
+      <c r="C92" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D92" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E92" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F92" s="37" t="inlineStr"/>
+    </row>
+    <row r="93" ht="18" customHeight="1">
+      <c r="A93" s="38" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="39" t="inlineStr">
+        <is>
+          <t>perioral dermatitis vs rosacea</t>
+        </is>
+      </c>
+      <c r="C93" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D93" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E93" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F93" s="43" t="inlineStr"/>
+    </row>
+    <row r="94" ht="18" customHeight="1">
+      <c r="A94" s="32" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="33" t="inlineStr">
+        <is>
+          <t>fungal acne</t>
+        </is>
+      </c>
+      <c r="C94" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D94" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E94" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F94" s="37" t="inlineStr"/>
+    </row>
+    <row r="95" ht="18" customHeight="1">
+      <c r="A95" s="38" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="39" t="inlineStr">
+        <is>
+          <t>malassezia folliculitis</t>
+        </is>
+      </c>
+      <c r="C95" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D95" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E95" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F95" s="43" t="inlineStr"/>
+    </row>
+    <row r="96" ht="18" customHeight="1">
+      <c r="A96" s="32" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="33" t="inlineStr">
+        <is>
+          <t>fungal acne vs regular acne</t>
+        </is>
+      </c>
+      <c r="C96" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D96" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E96" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F96" s="37" t="inlineStr"/>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="38" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="39" t="inlineStr">
+        <is>
+          <t>fungal acne safe moisturizer</t>
+        </is>
+      </c>
+      <c r="C97" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D97" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E97" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F97" s="43" t="inlineStr"/>
+    </row>
+    <row r="98" ht="18" customHeight="1">
+      <c r="A98" s="32" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="33" t="inlineStr">
+        <is>
+          <t>how to treat fungal acne</t>
+        </is>
+      </c>
+      <c r="C98" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D98" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E98" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F98" s="37" t="inlineStr"/>
+    </row>
+    <row r="99" ht="18" customHeight="1">
+      <c r="A99" s="38" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="39" t="inlineStr">
+        <is>
+          <t>fungal acne skincare routine</t>
+        </is>
+      </c>
+      <c r="C99" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D99" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E99" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F99" s="43" t="inlineStr"/>
+    </row>
+    <row r="100" ht="18" customHeight="1">
+      <c r="A100" s="32" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="33" t="inlineStr">
+        <is>
+          <t>sensitive skin vs damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C100" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D100" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E100" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F100" s="37" t="inlineStr"/>
+    </row>
+    <row r="101" ht="18" customHeight="1">
+      <c r="A101" s="38" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="39" t="inlineStr">
+        <is>
+          <t>how to know if skin is sensitive</t>
+        </is>
+      </c>
+      <c r="C101" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D101" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E101" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F101" s="43" t="inlineStr"/>
+    </row>
+    <row r="102" ht="18" customHeight="1">
+      <c r="A102" s="32" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" s="33" t="inlineStr">
+        <is>
+          <t>best moisturizer for sensitive skin</t>
+        </is>
+      </c>
+      <c r="C102" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D102" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E102" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F102" s="37" t="inlineStr"/>
+    </row>
+    <row r="103" ht="18" customHeight="1">
+      <c r="A103" s="38" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" s="39" t="inlineStr">
+        <is>
+          <t>sensitive skin routine</t>
+        </is>
+      </c>
+      <c r="C103" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D103" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E103" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F103" s="43" t="inlineStr"/>
+    </row>
+    <row r="104" ht="18" customHeight="1">
+      <c r="A104" s="32" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" s="33" t="inlineStr">
+        <is>
+          <t>non-irritating skincare sensitive skin</t>
+        </is>
+      </c>
+      <c r="C104" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D104" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E104" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F104" s="37" t="inlineStr"/>
+    </row>
+    <row r="105" ht="18" customHeight="1">
+      <c r="A105" s="38" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier repair acne prone skin</t>
+        </is>
+      </c>
+      <c r="C105" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D105" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E105" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F105" s="43" t="inlineStr"/>
+    </row>
+    <row r="106" ht="18" customHeight="1">
+      <c r="A106" s="32" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" s="33" t="inlineStr">
+        <is>
+          <t>does acne damage skin barrier</t>
+        </is>
+      </c>
+      <c r="C106" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D106" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E106" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F106" s="37" t="inlineStr"/>
+    </row>
+    <row r="107" ht="18" customHeight="1">
+      <c r="A107" s="38" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" s="39" t="inlineStr">
+        <is>
+          <t>non-comedogenic barrier repair moisturizer</t>
+        </is>
+      </c>
+      <c r="C107" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D107" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E107" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F107" s="43" t="inlineStr"/>
+    </row>
+    <row r="108" ht="18" customHeight="1">
+      <c r="A108" s="32" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" s="33" t="inlineStr">
+        <is>
+          <t>barrier repair routine for acne</t>
+        </is>
+      </c>
+      <c r="C108" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D108" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E108" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F108" s="37" t="inlineStr"/>
+    </row>
+    <row r="109" ht="18" customHeight="1">
+      <c r="A109" s="38" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" s="39" t="inlineStr">
+        <is>
+          <t>best moisturizer for acne and dry skin</t>
+        </is>
+      </c>
+      <c r="C109" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D109" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E109" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F109" s="43" t="inlineStr"/>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="32" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" s="33" t="inlineStr">
+        <is>
+          <t>CeraVe vs Cetaphil</t>
+        </is>
+      </c>
+      <c r="C110" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D110" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E110" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F110" s="37" t="inlineStr">
+        <is>
+          <t>Very high volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="18" customHeight="1">
+      <c r="A111" s="38" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" s="39" t="inlineStr">
+        <is>
+          <t>CeraVe vs Cetaphil for eczema</t>
+        </is>
+      </c>
+      <c r="C111" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D111" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E111" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F111" s="43" t="inlineStr"/>
+    </row>
+    <row r="112" ht="18" customHeight="1">
+      <c r="A112" s="32" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" s="33" t="inlineStr">
+        <is>
+          <t>CeraVe vs Cetaphil sensitive skin</t>
+        </is>
+      </c>
+      <c r="C112" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D112" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E112" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F112" s="37" t="inlineStr"/>
+    </row>
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="38" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" s="39" t="inlineStr">
+        <is>
+          <t>niacinamide vs vitamin C</t>
+        </is>
+      </c>
+      <c r="C113" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D113" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E113" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F113" s="43" t="inlineStr"/>
+    </row>
+    <row r="114" ht="18" customHeight="1">
+      <c r="A114" s="32" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" s="33" t="inlineStr">
+        <is>
+          <t>can you mix niacinamide and vitamin C</t>
+        </is>
+      </c>
+      <c r="C114" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D114" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E114" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F114" s="37" t="inlineStr"/>
+    </row>
+    <row r="115" ht="18" customHeight="1">
+      <c r="A115" s="38" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="39" t="inlineStr">
+        <is>
+          <t>hyaluronic acid vs glycerin moisturizer</t>
+        </is>
+      </c>
+      <c r="C115" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D115" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E115" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F115" s="43" t="inlineStr"/>
+    </row>
+    <row r="116" ht="18" customHeight="1">
+      <c r="A116" s="32" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="33" t="inlineStr">
+        <is>
+          <t>Cicaplast B5 vs CeraVe</t>
+        </is>
+      </c>
+      <c r="C116" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D116" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E116" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F116" s="37" t="inlineStr"/>
+    </row>
+    <row r="117" ht="18" customHeight="1">
+      <c r="A117" s="38" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="39" t="inlineStr">
+        <is>
+          <t>Paula's Choice vs CeraVe</t>
+        </is>
+      </c>
+      <c r="C117" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D117" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E117" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F117" s="43" t="inlineStr"/>
+    </row>
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="32" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="33" t="inlineStr">
+        <is>
+          <t>CeraVe Moisturizing Cream review</t>
+        </is>
+      </c>
+      <c r="C118" s="50" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D118" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E118" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F118" s="37" t="inlineStr"/>
+    </row>
+    <row r="119" ht="18" customHeight="1">
+      <c r="A119" s="38" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="39" t="inlineStr">
+        <is>
+          <t>La Roche-Posay Cicaplast review</t>
+        </is>
+      </c>
+      <c r="C119" s="51" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D119" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E119" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F119" s="43" t="inlineStr"/>
+    </row>
+    <row r="120" ht="18" customHeight="1">
+      <c r="A120" s="32" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="33" t="inlineStr">
+        <is>
+          <t>Paula's Choice Barrier Repair review</t>
+        </is>
+      </c>
+      <c r="C120" s="50" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D120" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E120" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F120" s="37" t="inlineStr"/>
+    </row>
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="38" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="39" t="inlineStr">
+        <is>
+          <t>The Ordinary NMF review</t>
+        </is>
+      </c>
+      <c r="C121" s="51" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D121" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E121" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F121" s="43" t="inlineStr"/>
+    </row>
+    <row r="122" ht="18" customHeight="1">
+      <c r="A122" s="32" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="33" t="inlineStr">
+        <is>
+          <t>Vanicream Gentle Cleanser review</t>
+        </is>
+      </c>
+      <c r="C122" s="50" t="inlineStr">
+        <is>
+          <t>Navigational</t>
+        </is>
+      </c>
+      <c r="D122" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E122" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F122" s="37" t="inlineStr"/>
+    </row>
+    <row r="123" ht="18" customHeight="1">
+      <c r="A123" s="38" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="39" t="inlineStr">
+        <is>
+          <t>best barrier repair moisturizer 2026</t>
+        </is>
+      </c>
+      <c r="C123" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D123" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E123" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F123" s="43" t="inlineStr"/>
+    </row>
+    <row r="124" ht="18" customHeight="1">
+      <c r="A124" s="32" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="33" t="inlineStr">
+        <is>
+          <t>best cleanser for damaged skin barrier</t>
+        </is>
+      </c>
+      <c r="C124" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D124" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E124" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F124" s="37" t="inlineStr"/>
+    </row>
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="38" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="39" t="inlineStr">
+        <is>
+          <t>gentle cleanser sensitive skin</t>
+        </is>
+      </c>
+      <c r="C125" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D125" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E125" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F125" s="43" t="inlineStr"/>
+    </row>
+    <row r="126" ht="18" customHeight="1">
+      <c r="A126" s="32" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="33" t="inlineStr">
+        <is>
+          <t>sulfate-free cleanser barrier repair</t>
+        </is>
+      </c>
+      <c r="C126" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D126" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E126" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F126" s="37" t="inlineStr"/>
+    </row>
+    <row r="127" ht="18" customHeight="1">
+      <c r="A127" s="38" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="39" t="inlineStr">
+        <is>
+          <t>non-stripping face wash</t>
+        </is>
+      </c>
+      <c r="C127" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D127" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E127" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F127" s="43" t="inlineStr"/>
+    </row>
+    <row r="128" ht="18" customHeight="1">
+      <c r="A128" s="32" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="33" t="inlineStr">
+        <is>
+          <t>best face wash dry damaged skin</t>
+        </is>
+      </c>
+      <c r="C128" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D128" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E128" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F128" s="37" t="inlineStr"/>
+    </row>
+    <row r="129" ht="18" customHeight="1">
+      <c r="A129" s="38" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="39" t="inlineStr">
+        <is>
+          <t>skin microbiome</t>
+        </is>
+      </c>
+      <c r="C129" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D129" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E129" s="52" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F129" s="43" t="inlineStr">
+        <is>
+          <t>Adjacent cluster</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="32" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="33" t="inlineStr">
+        <is>
+          <t>skin pH balance</t>
+        </is>
+      </c>
+      <c r="C130" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D130" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E130" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F130" s="37" t="inlineStr">
+        <is>
+          <t>Supporting concept</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="18" customHeight="1">
+      <c r="A131" s="38" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="39" t="inlineStr">
+        <is>
+          <t>acid mantle skin</t>
+        </is>
+      </c>
+      <c r="C131" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D131" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E131" s="52" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F131" s="43" t="inlineStr">
+        <is>
+          <t>Supporting concept</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="18" customHeight="1">
+      <c r="A132" s="32" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="33" t="inlineStr">
+        <is>
+          <t>what is the acid mantle</t>
+        </is>
+      </c>
+      <c r="C132" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D132" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E132" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F132" s="37" t="inlineStr"/>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="38" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="39" t="inlineStr">
+        <is>
+          <t>stratum corneum</t>
+        </is>
+      </c>
+      <c r="C133" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D133" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E133" s="52" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F133" s="43" t="inlineStr">
+        <is>
+          <t>Technical term</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="18" customHeight="1">
+      <c r="A134" s="32" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="33" t="inlineStr">
+        <is>
+          <t>corneum repair</t>
+        </is>
+      </c>
+      <c r="C134" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D134" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E134" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F134" s="37" t="inlineStr"/>
+    </row>
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="38" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier lipids</t>
+        </is>
+      </c>
+      <c r="C135" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D135" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E135" s="52" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F135" s="43" t="inlineStr"/>
+    </row>
+    <row r="136" ht="18" customHeight="1">
+      <c r="A136" s="32" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="33" t="inlineStr">
+        <is>
+          <t>epidermal barrier function</t>
+        </is>
+      </c>
+      <c r="C136" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D136" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E136" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F136" s="37" t="inlineStr">
+        <is>
+          <t>Clinical term</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="38" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier genes</t>
+        </is>
+      </c>
+      <c r="C137" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D137" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E137" s="52" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F137" s="43" t="inlineStr">
+        <is>
+          <t>Low competition niche</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="18" customHeight="1">
+      <c r="A138" s="32" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="33" t="inlineStr">
+        <is>
+          <t>filaggrin skin barrier</t>
+        </is>
+      </c>
+      <c r="C138" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D138" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E138" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F138" s="37" t="inlineStr">
+        <is>
+          <t>Genetic/clinical</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="18" customHeight="1">
+      <c r="A139" s="38" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="39" t="inlineStr">
+        <is>
+          <t>hot water skin barrier damage</t>
+        </is>
+      </c>
+      <c r="C139" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D139" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E139" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F139" s="43" t="inlineStr"/>
+    </row>
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="32" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="33" t="inlineStr">
+        <is>
+          <t>does washing face too much damage skin</t>
+        </is>
+      </c>
+      <c r="C140" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D140" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E140" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F140" s="37" t="inlineStr"/>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="38" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="39" t="inlineStr">
+        <is>
+          <t>stress skin barrier</t>
+        </is>
+      </c>
+      <c r="C141" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D141" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E141" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F141" s="43" t="inlineStr"/>
+    </row>
+    <row r="142" ht="18" customHeight="1">
+      <c r="A142" s="32" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="33" t="inlineStr">
+        <is>
+          <t>alcohol in skincare skin barrier</t>
+        </is>
+      </c>
+      <c r="C142" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D142" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E142" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F142" s="37" t="inlineStr"/>
+    </row>
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="38" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="39" t="inlineStr">
+        <is>
+          <t>fragrance free skincare sensitive skin</t>
+        </is>
+      </c>
+      <c r="C143" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D143" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E143" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F143" s="43" t="inlineStr"/>
+    </row>
+    <row r="144" ht="18" customHeight="1">
+      <c r="A144" s="32" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="33" t="inlineStr">
+        <is>
+          <t>does diet affect skin barrier</t>
+        </is>
+      </c>
+      <c r="C144" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D144" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E144" s="34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F144" s="37" t="inlineStr"/>
+    </row>
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="38" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="39" t="inlineStr">
+        <is>
+          <t>omega 3 for skin barrier</t>
+        </is>
+      </c>
+      <c r="C145" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D145" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E145" s="40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="F145" s="43" t="inlineStr"/>
+    </row>
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="32" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="33" t="inlineStr">
+        <is>
+          <t>sleep and skin barrier repair</t>
+        </is>
+      </c>
+      <c r="C146" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D146" s="35" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E146" s="53" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="F146" s="37" t="inlineStr"/>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="38" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="39" t="inlineStr">
+        <is>
+          <t>skin barrier 101</t>
+        </is>
+      </c>
+      <c r="C147" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D147" s="41" t="inlineStr">
+        <is>
+          <t>Top</t>
+        </is>
+      </c>
+      <c r="E147" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F147" s="43" t="inlineStr">
+        <is>
+          <t>Exact-match pillar title</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="18" customHeight="1">
+      <c r="A148" s="32" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="33" t="inlineStr">
+        <is>
+          <t>barrier cream for face</t>
+        </is>
+      </c>
+      <c r="C148" s="47" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D148" s="48" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E148" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F148" s="37" t="inlineStr"/>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="A149" s="38" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="39" t="inlineStr">
+        <is>
+          <t>best moisturizer for dry damaged skin</t>
+        </is>
+      </c>
+      <c r="C149" s="46" t="inlineStr">
+        <is>
+          <t>Commercial</t>
+        </is>
+      </c>
+      <c r="D149" s="49" t="inlineStr">
+        <is>
+          <t>Bottom</t>
+        </is>
+      </c>
+      <c r="E149" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F149" s="43" t="inlineStr"/>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="A150" s="32" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="33" t="inlineStr">
+        <is>
+          <t>skin barrier ingredients to avoid</t>
+        </is>
+      </c>
+      <c r="C150" s="34" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D150" s="44" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E150" s="36" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F150" s="37" t="inlineStr">
+        <is>
+          <t>Negative-intent high CTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="A151" s="38" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="39" t="inlineStr">
+        <is>
+          <t>repair skin barrier overnight</t>
+        </is>
+      </c>
+      <c r="C151" s="40" t="inlineStr">
+        <is>
+          <t>Informational</t>
+        </is>
+      </c>
+      <c r="D151" s="45" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="E151" s="42" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="F151" s="43" t="inlineStr">
+        <is>
+          <t>Urgency intent</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>